<commit_message>
feat(F-NAR-019): TREE-COL-010 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-010.xlsx
+++ b/stories/arbres/TREE-COL-010.xlsx
@@ -2734,17 +2734,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
+          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
+          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2887,7 +2887,7 @@
 papa|On peut en ajouter.
 enfant-f|Celle-là aussi.
 narrateur|Les autres suivent, une par une.
-maman|Chaque clic a eu sa place.
+maman|Le clic est net, cette fois.
 narrateur|Les oranges rejoignent le petit panier.
 enfant-f|Il n'est plus vide.</t>
         </is>
@@ -3484,17 +3484,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
+          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
+          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3632,7 +3632,7 @@
 narrateur|Mila prend le torchon rayé.
 narrateur|Papa approche une orange trop vite.
 enfant-f|Pas maintenant.
-narrateur|Elle essuie, puis elle attend.
+narrateur|Elle essuie, puis elle regarde.
 narrateur|Le métal redevient mat.
 enfant-f|C'est sec.
 papa|On pose les oranges.
@@ -4434,17 +4434,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as demandée au bon silence. Le jus de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.</t>
+          <t>L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as dite après le thym. Le jus de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as demandée au bon silence. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as dite après le thym. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as demandée au bon silence. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'orange du fond trône dans le panier. Les autres attendent près de l'évier. Celle-là, d'abord. Tu l'as dite après le thym. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; de celle du fond est plus pâle. On la reconnaît ? Oui. Elle était cachée. Une écharde de caisse reste dans l'osier. L'orange du fond brille toute seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4585,7 +4585,7 @@
           <t>narrateur|L'orange du fond trône dans le panier.
 narrateur|Les autres attendent près de l'évier.
 enfant-f|Celle-là, d'abord.
-maman|Tu l'as demandée au bon silence.
+maman|Tu l'as dite après le thym.
 narrateur|Le jus de celle du fond est plus pâle.
 papa|On la reconnaît ?
 enfant-f|Oui.
@@ -4623,17 +4623,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
+          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
+          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4773,7 +4773,7 @@
 narrateur|Le compte se casse.
 narrateur|Elle remet le fruit dans la caisse.
 narrateur|Les nombres reprennent.
-enfant-f|J'attends la fin.
+enfant-f|Les nombres d'abord.
 papa|Le tas est le sien, maintenant.
 maman|Quatre, comme elle voulait.
 narrateur|Le bois de la caisse sent l'écorce.
@@ -5373,17 +5373,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le panier dans le chariot. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. Tu as parlé au bon moment.</t>
+          <t>Mila pose le panier dans le chariot. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. On voit la balance.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila pose le panier dans le &lt;emphasis level="moderate"&gt;chariot&lt;/emphasis&gt;. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. Tu as parlé au bon moment.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila pose le panier dans le &lt;emphasis level="moderate"&gt;chariot&lt;/emphasis&gt;. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. On voit la balance.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Mila pose le panier dans le &lt;emphasis&gt;chariot&lt;/emphasis&gt;. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. Tu as parlé au bon moment.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila pose le panier dans le &lt;emphasis&gt;chariot&lt;/emphasis&gt;. La roue tient le tapis du stand. Papa tire, maman paie des fraises. Deux gestes en même temps. Le panier glisse vers le bord. Mila l'attrape, sans crier. Maman range la monnaie. Le panier allait tomber. On recule le chariot, alors. La roue quitte le tapis. La balance reparaît. On voit la balance.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5532,7 +5532,7 @@
 papa|On recule le chariot, alors.
 narrateur|La roue quitte le tapis.
 narrateur|La balance reparaît.
-maman|Tu as parlé au bon moment.</t>
+maman|On voit la balance.</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr">
@@ -5948,17 +5948,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. J'ai attendu qu'elle s'arrête. Le jus de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.</t>
+          <t>Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. Elle ne roulait plus. Le jus de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. J'ai attendu qu'elle s'arrête. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. Elle ne roulait plus. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. J'ai attendu qu'elle s'arrête. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le panier a voyagé dans le chariot. Il pose près de la fenêtre. La première orange n'a pas bougé. Elle s'est calée, toute seule. Elle ne roulait plus. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; de celle-là, pour toi. Dehors, une roue lointaine se tait. Mila boit, les yeux sur le panier. Dans l'osier, la première orange tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6100,7 +6100,7 @@
 narrateur|Il pose près de la fenêtre.
 narrateur|La première orange n'a pas bougé.
 papa|Elle s'est calée, toute seule.
-enfant-f|J'ai attendu qu'elle s'arrête.
+enfant-f|Elle ne roulait plus.
 maman|Le jus de celle-là, pour toi.
 narrateur|Dehors, une roue lointaine se tait.
 narrateur|Mila boit, les yeux sur le panier.
@@ -6136,17 +6136,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
+          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
+          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6285,7 +6285,7 @@
 enfant-f|Elles partent !
 narrateur|Papa parle du chemin du retour.
 narrateur|Il n'a pas vu la roue.
-narrateur|Mila attend sa fin de phrase.
+narrateur|Mila laisse papa finir.
 enfant-f|Le tas va vers la roue.
 papa|On les recule, alors.
 narrateur|Le tas se cale contre le bois.
@@ -6512,17 +6512,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges rejoignent le petit panier. Il n'est plus vide. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6664,7 +6664,7 @@
 narrateur|Papa n'entend pas, il charge.
 narrateur|Mila montre le torchon sale.
 papa|Pardon.
-papa|J'attendais pas.
+papa|Je chargeais trop vite.
 narrateur|Elle finit le fond, toute seule.
 maman|Les oranges peuvent entrer, là.
 narrateur|Les oranges rejoignent le petit panier.
@@ -8031,17 +8031,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges glissent dans le filet. Les mailles tiennent.</t>
+          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges glissent dans le filet. Les mailles tiennent.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
+          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8184,7 +8184,7 @@
 papa|On peut en ajouter.
 enfant-f|Celle-là aussi.
 narrateur|Les autres suivent, une par une.
-maman|Chaque clic a eu sa place.
+maman|Le clic est net, cette fois.
 narrateur|Les oranges glissent dans le filet.
 enfant-f|Les mailles tiennent.</t>
         </is>
@@ -8781,17 +8781,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent.</t>
+          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
+          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8929,7 +8929,7 @@
 narrateur|Mila prend le torchon rayé.
 narrateur|Papa approche une orange trop vite.
 enfant-f|Pas maintenant.
-narrateur|Elle essuie, puis elle attend.
+narrateur|Elle essuie, puis elle regarde.
 narrateur|Le métal redevient mat.
 enfant-f|C'est sec.
 papa|On pose les oranges.
@@ -9156,17 +9156,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Une maille du filet pince une latte. Mila tire, la caisse crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Elle attend la fin des mots. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.</t>
+          <t>Une maille du filet pince une latte. Mila tire, la caisse crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Les mots de thym s'arrêtent. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Une maille du filet pince une latte. Mila tire, la &lt;emphasis level="moderate"&gt;caisse&lt;/emphasis&gt; crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Elle attend la fin des mots. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Une maille du filet pince une latte. Mila tire, la &lt;emphasis level="moderate"&gt;caisse&lt;/emphasis&gt; crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Les mots de thym s'arrêtent. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Une maille du filet pince une latte. Mila tire, la &lt;emphasis&gt;caisse&lt;/emphasis&gt; crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Elle attend la fin des mots. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Une maille du filet pince une latte. Mila tire, la &lt;emphasis&gt;caisse&lt;/emphasis&gt; crisse. La marchande décrit le thym à maman. Il est coincé ! Les deux voix couvrent la sienne. Mila lâche la maille. Les mots de thym s'arrêtent. Le thym est choisi. La marchande se tait. Le filet tenait la caisse. On le détache ensemble. L'orange du fond apparaît.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9310,7 +9310,7 @@
 enfant-f|Il est coincé !
 narrateur|Les deux voix couvrent la sienne.
 narrateur|Mila lâche la maille.
-narrateur|Elle attend la fin des mots.
+narrateur|Les mots de thym s'arrêtent.
 narrateur|Le thym est choisi.
 narrateur|La marchande se tait.
 enfant-f|Le filet tenait la caisse.
@@ -9920,17 +9920,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent.</t>
+          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
+          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10070,7 +10070,7 @@
 narrateur|Le compte se casse.
 narrateur|Elle remet le fruit dans la caisse.
 narrateur|Les nombres reprennent.
-enfant-f|J'attends la fin.
+enfant-f|Les nombres d'abord.
 papa|Le tas est le sien, maintenant.
 maman|Quatre, comme elle voulait.
 narrateur|Le bois de la caisse sent l'écorce.
@@ -11245,17 +11245,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. J'ai attendu le choc. Le jus, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.</t>
+          <t>Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. Le choc, puis plus rien. Le jus, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. J'ai attendu le choc. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt;, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. Le choc, puis plus rien. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt;, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. J'ai attendu le choc. Le &lt;emphasis&gt;jus&lt;/emphasis&gt;, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le filet repose sur le rebord du chariot. Le chariot est rentré dans la cour. Mila prend la première orange. Celle qui ne roulait plus. Le choc, puis plus rien. Le &lt;emphasis&gt;jus&lt;/emphasis&gt;, sur le pas ? Ils s'assoient sur la pierre froide. Le filet pend dans la lumière. La première orange a un goût de vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11397,7 +11397,7 @@
 narrateur|Le chariot est rentré dans la cour.
 narrateur|Mila prend la première orange.
 papa|Celle qui ne roulait plus.
-enfant-f|J'ai attendu le choc.
+enfant-f|Le choc, puis plus rien.
 maman|Le jus, sur le pas ?
 narrateur|Ils s'assoient sur la pierre froide.
 narrateur|Le filet pend dans la lumière.
@@ -11433,17 +11433,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent.</t>
+          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
+          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11582,7 +11582,7 @@
 enfant-f|Elles partent !
 narrateur|Papa parle du chemin du retour.
 narrateur|Il n'a pas vu la roue.
-narrateur|Mila attend sa fin de phrase.
+narrateur|Mila laisse papa finir.
 enfant-f|Le tas va vers la roue.
 papa|On les recule, alors.
 narrateur|Le tas se cale contre le bois.
@@ -11808,17 +11808,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent.</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Les oranges glissent dans le filet. Les mailles tiennent. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11960,7 +11960,7 @@
 narrateur|Papa n'entend pas, il charge.
 narrateur|Mila montre le torchon sale.
 papa|Pardon.
-papa|J'attendais pas.
+papa|Je chargeais trop vite.
 narrateur|Elle finit le fond, toute seule.
 maman|Les oranges peuvent entrer, là.
 narrateur|Les oranges glissent dans le filet.
@@ -13325,17 +13325,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
+          <t>Mila pose une seule orange. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila pose une seule &lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Chaque clic a eu sa place. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
+          <t>Mila pose une seule &lt;emphasis&gt;orange&lt;/emphasis&gt;. Sa main revient avec une deuxième. L'aiguille n'a pas fini de bouger. Elle retire la deuxième orange. La balance fait clic. L'aiguille s'arrête. On peut en ajouter. Celle-là aussi. Les autres suivent, une par une. Le clic est net, cette fois. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13478,7 +13478,7 @@
 papa|On peut en ajouter.
 enfant-f|Celle-là aussi.
 narrateur|Les autres suivent, une par une.
-maman|Chaque clic a eu sa place.
+maman|Le clic est net, cette fois.
 narrateur|Mila tend la pièce, sans la secouer.
 enfant-f|Pour les oranges rondes.</t>
         </is>
@@ -14076,17 +14076,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
+          <t>Le plateau reste collant de pomme. Mila prend le torchon rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau reste collant de pomme. Mila prend le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle attend. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
+          <t>Le plateau reste collant de pomme. Mila prend le &lt;emphasis&gt;torchon&lt;/emphasis&gt; rayé. Papa approche une orange trop vite. Pas maintenant. Elle essuie, puis elle regarde. Le métal redevient mat. C'est sec. On pose les oranges. Le premier clic sonne net. Le torchon a rendu le plateau. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14224,7 +14224,7 @@
 narrateur|Mila prend le torchon rayé.
 narrateur|Papa approche une orange trop vite.
 enfant-f|Pas maintenant.
-narrateur|Elle essuie, puis elle attend.
+narrateur|Elle essuie, puis elle regarde.
 narrateur|Le métal redevient mat.
 enfant-f|C'est sec.
 papa|On pose les oranges.
@@ -14263,17 +14263,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal a attendu, lui aussi. Le jus tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.</t>
+          <t>La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal était prêt, lui aussi. Le jus tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal a attendu, lui aussi. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal était prêt, lui aussi. Le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal a attendu, lui aussi. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La pièce sèche sur le torchon rayé. Mila presse, les doigts propres. Plus de pomme, plus de collant. J'ai dit : pas maintenant. Le métal était prêt, lui aussi. Le &lt;emphasis&gt;jus&lt;/emphasis&gt; tombe dans un bol à fleurs. La pièce ne glisse plus. Une rayure du torchon brille, humide. Le bol sent l'orange chaude.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14415,7 +14415,7 @@
 narrateur|Mila presse, les doigts propres.
 papa|Plus de pomme, plus de collant.
 enfant-f|J'ai dit : pas maintenant.
-maman|Le métal a attendu, lui aussi.
+maman|Le métal était prêt, lui aussi.
 narrateur|Le jus tombe dans un bol à fleurs.
 narrateur|La pièce ne glisse plus.
 narrateur|Une rayure du torchon brille, humide.
@@ -15214,17 +15214,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
+          <t>La marchande ramasse un tas. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La marchande ramasse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. J'attends la fin. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
+          <t>La marchande ramasse un &lt;emphasis&gt;tas&lt;/emphasis&gt;. Elle compte à voix haute. Mila ajoute une orange au milieu. Le compte se casse. Elle remet le fruit dans la caisse. Les nombres reprennent. Les nombres d'abord. Le tas est le sien, maintenant. Quatre, comme elle voulait. Le bois de la caisse sent l'écorce. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15364,7 +15364,7 @@
 narrateur|Le compte se casse.
 narrateur|Elle remet le fruit dans la caisse.
 narrateur|Les nombres reprennent.
-enfant-f|J'attends la fin.
+enfant-f|Les nombres d'abord.
 papa|Le tas est le sien, maintenant.
 maman|Quatre, comme elle voulait.
 narrateur|Le bois de la caisse sent l'écorce.
@@ -15965,17 +15965,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>La pièce roule sous le chariot. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. Elle attend la monnaie rangée. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci d'avoir attendu le moment.</t>
+          <t>La pièce roule sous le chariot. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. La monnaie rejoint la poche. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci, la pièce est là.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La pièce roule sous le &lt;emphasis level="moderate"&gt;chariot&lt;/emphasis&gt;. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. Elle attend la monnaie rangée. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci d'avoir attendu le moment.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La pièce roule sous le &lt;emphasis level="moderate"&gt;chariot&lt;/emphasis&gt;. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. La monnaie rejoint la poche. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci, la pièce est là.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La pièce roule sous le &lt;emphasis&gt;chariot&lt;/emphasis&gt;. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. Elle attend la monnaie rangée. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci d'avoir attendu le moment.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La pièce roule sous le &lt;emphasis&gt;chariot&lt;/emphasis&gt;. Elle est dessous ! Papa veut pousser pour chercher. Maman tend l'argent des fraises. La roue pourrait bouger. Mila recule les mains. La monnaie rejoint la poche. La pièce est sous le chariot. On ne touche pas la roue. Il se baisse, le chariot immobile. La pièce reparaît, un peu poussiéreuse. Merci, la pièce est là.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -16119,12 +16119,12 @@
 narrateur|Maman tend l'argent des fraises.
 narrateur|La roue pourrait bouger.
 narrateur|Mila recule les mains.
-narrateur|Elle attend la monnaie rangée.
+narrateur|La monnaie rejoint la poche.
 enfant-f|La pièce est sous le chariot.
 papa|On ne touche pas la roue.
 narrateur|Il se baisse, le chariot immobile.
 narrateur|La pièce reparaît, un peu poussiéreuse.
-maman|Merci d'avoir attendu le moment.</t>
+maman|Merci, la pièce est là.</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr">
@@ -16728,17 +16728,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
+          <t>Mila verse un tas dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila verse un &lt;emphasis level="moderate"&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila attend sa fin de phrase. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
+          <t>Mila verse un &lt;emphasis&gt;tas&lt;/emphasis&gt; dans le chariot. Les oranges roulent vers la roue. Elles partent ! Papa parle du chemin du retour. Il n'a pas vu la roue. Mila laisse papa finir. Le tas va vers la roue. On les recule, alors. Le tas se cale contre le bois. Plus rien ne roule. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16877,7 +16877,7 @@
 enfant-f|Elles partent !
 narrateur|Papa parle du chemin du retour.
 narrateur|Il n'a pas vu la roue.
-narrateur|Mila attend sa fin de phrase.
+narrateur|Mila laisse papa finir.
 enfant-f|Le tas va vers la roue.
 papa|On les recule, alors.
 narrateur|Le tas se cale contre le bois.
@@ -16915,17 +16915,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le tas cache la pièce au fond du bol. Mila verse le jus par-dessus. Elles allaient vers la roue. J'ai attendu ta phrase. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.</t>
+          <t>Le tas cache la pièce au fond du bol. Mila verse le jus par-dessus. Elles allaient vers la roue. Après tes mots, je l'ai dit. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le tas cache la pièce au fond du bol. Mila verse le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; par-dessus. Elles allaient vers la roue. J'ai attendu ta phrase. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le tas cache la pièce au fond du bol. Mila verse le &lt;emphasis level="moderate"&gt;jus&lt;/emphasis&gt; par-dessus. Elles allaient vers la roue. Après tes mots, je l'ai dit. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le tas cache la pièce au fond du bol. Mila verse le &lt;emphasis&gt;jus&lt;/emphasis&gt; par-dessus. Elles allaient vers la roue. J'ai attendu ta phrase. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le tas cache la pièce au fond du bol. Mila verse le &lt;emphasis&gt;jus&lt;/emphasis&gt; par-dessus. Elles allaient vers la roue. Après tes mots, je l'ai dit. On retrouve la pièce après ? Mila plonge deux doigts, puis sourit. Elle est là, collée. Ils la lavent sous l'eau froide. Le tas, lui, a fini en jus doré.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -17066,7 +17066,7 @@
           <t>narrateur|Le tas cache la pièce au fond du bol.
 narrateur|Mila verse le jus par-dessus.
 papa|Elles allaient vers la roue.
-enfant-f|J'ai attendu ta phrase.
+enfant-f|Après tes mots, je l'ai dit.
 maman|On retrouve la pièce après ?
 narrateur|Mila plonge deux doigts, puis sourit.
 enfant-f|Elle est là, collée.
@@ -17103,17 +17103,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le torchon. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis level="moderate"&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. J'attendais pas. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
+          <t>Le fond du chariot porte du sable. Mila essuie avec le &lt;emphasis&gt;torchon&lt;/emphasis&gt;. Papa pose une orange trop tôt. Le fruit frotte le grain. Le sable. Papa n'entend pas, il charge. Mila montre le torchon sale. Pardon. Je chargeais trop vite. Elle finit le fond, toute seule. Les oranges peuvent entrer, là. Mila tend la pièce, sans la secouer. Pour les oranges rondes. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17255,7 +17255,7 @@
 narrateur|Papa n'entend pas, il charge.
 narrateur|Mila montre le torchon sale.
 papa|Pardon.
-papa|J'attendais pas.
+papa|Je chargeais trop vite.
 narrateur|Elle finit le fond, toute seule.
 maman|Les oranges peuvent entrer, là.
 narrateur|Mila tend la pièce, sans la secouer.
@@ -17473,7 +17473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17530,6 +17530,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>